<commit_message>
Add Labs 3-5 and Lab 1 final notebook; ignore scratch files
- LAB_1: ds_lab1_final.ipynb (14/14 cells, clean), refreshed xlsx data, drop LAB_1.zip
- LAB_3: ds_3.ipynb
- LAB_4: ds_1.ipynb, ds_2.ipynb (clean)
- LAB_5: exp5 (1).ipynb (clean)
- gitignore: website/ build, _extract/_verify scripts, .hallmark log, zip archives
</commit_message>
<xml_diff>
--- a/LAB_1/college_data.xlsx
+++ b/LAB_1/college_data.xlsx
@@ -420,7 +420,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Rool_No</t>
+          <t>Roll_No</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3">
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>200</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5">
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>500</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>